<commit_message>
Update files on 2026-08-17
</commit_message>
<xml_diff>
--- a/src/test/resources/codechgfile.text.xlsx
+++ b/src/test/resources/codechgfile.text.xlsx
@@ -34,7 +34,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J904"/>
+  <dimension ref="A1:J876"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -45588,1462 +45588,6 @@
         </is>
       </c>
     </row>
-    <row r="877">
-      <c r="A877" t="inlineStr">
-        <is>
-          <t xml:space="preserve">변경    </t>
-        </is>
-      </c>
-      <c r="B877" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0120702</t>
-        </is>
-      </c>
-      <c r="C877" t="inlineStr">
-        <is>
-          <t xml:space="preserve">농축협　　　　　　　</t>
-        </is>
-      </c>
-      <c r="D877" t="inlineStr">
-        <is>
-          <t xml:space="preserve">인천옹진농협　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="E877" t="inlineStr">
-        <is>
-          <t xml:space="preserve">032  885  2001 </t>
-        </is>
-      </c>
-      <c r="F877" t="inlineStr">
-        <is>
-          <t xml:space="preserve">032  885  2006 </t>
-        </is>
-      </c>
-      <c r="G877" t="inlineStr">
-        <is>
-          <t xml:space="preserve">22331 </t>
-        </is>
-      </c>
-      <c r="H877" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20260716</t>
-        </is>
-      </c>
-      <c r="I877" t="inlineStr">
-        <is>
-          <t xml:space="preserve">인천광역시　제물포구　인중로４１번길　１　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="J877" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       </t>
-        </is>
-      </c>
-    </row>
-    <row r="878">
-      <c r="A878" t="inlineStr">
-        <is>
-          <t xml:space="preserve">변경    </t>
-        </is>
-      </c>
-      <c r="B878" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0141516</t>
-        </is>
-      </c>
-      <c r="C878" t="inlineStr">
-        <is>
-          <t xml:space="preserve">농축협　　　　　　　</t>
-        </is>
-      </c>
-      <c r="D878" t="inlineStr">
-        <is>
-          <t xml:space="preserve">서인천　율도　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="E878" t="inlineStr">
-        <is>
-          <t xml:space="preserve">032  578  8256 </t>
-        </is>
-      </c>
-      <c r="F878" t="inlineStr">
-        <is>
-          <t xml:space="preserve">032  578  8140 </t>
-        </is>
-      </c>
-      <c r="G878" t="inlineStr">
-        <is>
-          <t xml:space="preserve">22786 </t>
-        </is>
-      </c>
-      <c r="H878" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20260716</t>
-        </is>
-      </c>
-      <c r="I878" t="inlineStr">
-        <is>
-          <t xml:space="preserve">인천광역시　서해구　율도로　３２　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="J878" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       </t>
-        </is>
-      </c>
-    </row>
-    <row r="879">
-      <c r="A879" t="inlineStr">
-        <is>
-          <t xml:space="preserve">변경    </t>
-        </is>
-      </c>
-      <c r="B879" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0149589</t>
-        </is>
-      </c>
-      <c r="C879" t="inlineStr">
-        <is>
-          <t xml:space="preserve">농축협　　　　　　　</t>
-        </is>
-      </c>
-      <c r="D879" t="inlineStr">
-        <is>
-          <t xml:space="preserve">서인천　서곶　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="E879" t="inlineStr">
-        <is>
-          <t xml:space="preserve">032  561  9801 </t>
-        </is>
-      </c>
-      <c r="F879" t="inlineStr">
-        <is>
-          <t xml:space="preserve">032  561  9804 </t>
-        </is>
-      </c>
-      <c r="G879" t="inlineStr">
-        <is>
-          <t xml:space="preserve">22724 </t>
-        </is>
-      </c>
-      <c r="H879" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20260716</t>
-        </is>
-      </c>
-      <c r="I879" t="inlineStr">
-        <is>
-          <t xml:space="preserve">인천광역시　서해구　승학로　２５３　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="J879" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       </t>
-        </is>
-      </c>
-    </row>
-    <row r="880">
-      <c r="A880" t="inlineStr">
-        <is>
-          <t xml:space="preserve">변경    </t>
-        </is>
-      </c>
-      <c r="B880" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0151881</t>
-        </is>
-      </c>
-      <c r="C880" t="inlineStr">
-        <is>
-          <t xml:space="preserve">농축협　　　　　　　</t>
-        </is>
-      </c>
-      <c r="D880" t="inlineStr">
-        <is>
-          <t xml:space="preserve">목포원예　신도심　　　　　　　</t>
-        </is>
-      </c>
-      <c r="E880" t="inlineStr">
-        <is>
-          <t xml:space="preserve">061  283  6321 </t>
-        </is>
-      </c>
-      <c r="F880" t="inlineStr">
-        <is>
-          <t xml:space="preserve">061  283  4777 </t>
-        </is>
-      </c>
-      <c r="G880" t="inlineStr">
-        <is>
-          <t xml:space="preserve">58696 </t>
-        </is>
-      </c>
-      <c r="H880" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20260716</t>
-        </is>
-      </c>
-      <c r="I880" t="inlineStr">
-        <is>
-          <t xml:space="preserve">전남광주통합특별시　목포시　교육로４１번길　２５　　　　　　　　　　　　　　　　　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="J880" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       </t>
-        </is>
-      </c>
-    </row>
-    <row r="881">
-      <c r="A881" t="inlineStr">
-        <is>
-          <t xml:space="preserve">변경    </t>
-        </is>
-      </c>
-      <c r="B881" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0155395</t>
-        </is>
-      </c>
-      <c r="C881" t="inlineStr">
-        <is>
-          <t xml:space="preserve">농축협　　　　　　　</t>
-        </is>
-      </c>
-      <c r="D881" t="inlineStr">
-        <is>
-          <t xml:space="preserve">서인천　청라　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="E881" t="inlineStr">
-        <is>
-          <t xml:space="preserve">032  568  9320 </t>
-        </is>
-      </c>
-      <c r="F881" t="inlineStr">
-        <is>
-          <t xml:space="preserve">032  568  9321 </t>
-        </is>
-      </c>
-      <c r="G881" t="inlineStr">
-        <is>
-          <t xml:space="preserve">22737 </t>
-        </is>
-      </c>
-      <c r="H881" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20260716</t>
-        </is>
-      </c>
-      <c r="I881" t="inlineStr">
-        <is>
-          <t xml:space="preserve">인천광역시　서해구　중봉대로５８６번길　２２　청라엑슬루타워상가　Ｂ동２０６호　　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="J881" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       </t>
-        </is>
-      </c>
-    </row>
-    <row r="882">
-      <c r="A882" t="inlineStr">
-        <is>
-          <t xml:space="preserve">변경    </t>
-        </is>
-      </c>
-      <c r="B882" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0175346</t>
-        </is>
-      </c>
-      <c r="C882" t="inlineStr">
-        <is>
-          <t xml:space="preserve">농축협　　　　　　　</t>
-        </is>
-      </c>
-      <c r="D882" t="inlineStr">
-        <is>
-          <t xml:space="preserve">광주축산농협　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="E882" t="inlineStr">
-        <is>
-          <t xml:space="preserve">062  942  5885 </t>
-        </is>
-      </c>
-      <c r="F882" t="inlineStr">
-        <is>
-          <t xml:space="preserve">062  228  1080 </t>
-        </is>
-      </c>
-      <c r="G882" t="inlineStr">
-        <is>
-          <t xml:space="preserve">62380 </t>
-        </is>
-      </c>
-      <c r="H882" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20260716</t>
-        </is>
-      </c>
-      <c r="I882" t="inlineStr">
-        <is>
-          <t xml:space="preserve">전남광주통합특별시　광산구　상무대로　３１３　　　　　　　　　　　　　　　　　　　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="J882" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       </t>
-        </is>
-      </c>
-    </row>
-    <row r="883">
-      <c r="A883" t="inlineStr">
-        <is>
-          <t xml:space="preserve">변경    </t>
-        </is>
-      </c>
-      <c r="B883" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0175537</t>
-        </is>
-      </c>
-      <c r="C883" t="inlineStr">
-        <is>
-          <t xml:space="preserve">농축협　　　　　　　</t>
-        </is>
-      </c>
-      <c r="D883" t="inlineStr">
-        <is>
-          <t xml:space="preserve">순천광양　남부　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="E883" t="inlineStr">
-        <is>
-          <t xml:space="preserve">061  745  3700 </t>
-        </is>
-      </c>
-      <c r="F883" t="inlineStr">
-        <is>
-          <t xml:space="preserve">061  745  3747 </t>
-        </is>
-      </c>
-      <c r="G883" t="inlineStr">
-        <is>
-          <t xml:space="preserve">57962 </t>
-        </is>
-      </c>
-      <c r="H883" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20260716</t>
-        </is>
-      </c>
-      <c r="I883" t="inlineStr">
-        <is>
-          <t xml:space="preserve">전남광주통합특별시　순천시　풍덕주택길　２６　　　　　　　　　　　　　　　　　　　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="J883" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       </t>
-        </is>
-      </c>
-    </row>
-    <row r="884">
-      <c r="A884" t="inlineStr">
-        <is>
-          <t xml:space="preserve">잠정패쇄</t>
-        </is>
-      </c>
-      <c r="B884" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0184175</t>
-        </is>
-      </c>
-      <c r="C884" t="inlineStr">
-        <is>
-          <t xml:space="preserve">농축협　　　　　　　</t>
-        </is>
-      </c>
-      <c r="D884" t="inlineStr">
-        <is>
-          <t xml:space="preserve">대전충남양계　두성　　　　　　</t>
-        </is>
-      </c>
-      <c r="E884" t="inlineStr">
-        <is>
-          <t xml:space="preserve">041  622  6305 </t>
-        </is>
-      </c>
-      <c r="F884" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0503 8880 2628 </t>
-        </is>
-      </c>
-      <c r="G884" t="inlineStr">
-        <is>
-          <t xml:space="preserve">31112 </t>
-        </is>
-      </c>
-      <c r="H884" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20260716</t>
-        </is>
-      </c>
-      <c r="I884" t="inlineStr">
-        <is>
-          <t xml:space="preserve">충청남도　천안시　서북구　두정공원２길　２６　　　　　　　　　　　　　　　　　　　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="J884" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0173979</t>
-        </is>
-      </c>
-    </row>
-    <row r="885">
-      <c r="A885" t="inlineStr">
-        <is>
-          <t xml:space="preserve">신규    </t>
-        </is>
-      </c>
-      <c r="B885" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0508735</t>
-        </is>
-      </c>
-      <c r="C885" t="inlineStr">
-        <is>
-          <t xml:space="preserve">저축은행　　　　　　</t>
-        </is>
-      </c>
-      <c r="D885" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ＩＢＫ　　　종합금융４부　　　</t>
-        </is>
-      </c>
-      <c r="E885" t="inlineStr">
-        <is>
-          <t xml:space="preserve">051  791  4300 </t>
-        </is>
-      </c>
-      <c r="F885" t="inlineStr">
-        <is>
-          <t xml:space="preserve">051  791  4305 </t>
-        </is>
-      </c>
-      <c r="G885" t="inlineStr">
-        <is>
-          <t xml:space="preserve">47254 </t>
-        </is>
-      </c>
-      <c r="H885" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20260716</t>
-        </is>
-      </c>
-      <c r="I885" t="inlineStr">
-        <is>
-          <t xml:space="preserve">부산광역시　부산진구　중앙대로　７３５　（부전동）　３층　ＩＢＫ저축은행　　　　　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="J885" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       </t>
-        </is>
-      </c>
-    </row>
-    <row r="886">
-      <c r="A886" t="inlineStr">
-        <is>
-          <t xml:space="preserve">신규    </t>
-        </is>
-      </c>
-      <c r="B886" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0023676</t>
-        </is>
-      </c>
-      <c r="C886" t="inlineStr">
-        <is>
-          <t xml:space="preserve">산업　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="D886" t="inlineStr">
-        <is>
-          <t xml:space="preserve">서남권투자금융센터　　　　　　</t>
-        </is>
-      </c>
-      <c r="E886" t="inlineStr">
-        <is>
-          <t xml:space="preserve">062  958  1057 </t>
-        </is>
-      </c>
-      <c r="F886" t="inlineStr">
-        <is>
-          <t xml:space="preserve">062  531  6038 </t>
-        </is>
-      </c>
-      <c r="G886" t="inlineStr">
-        <is>
-          <t xml:space="preserve">62355 </t>
-        </is>
-      </c>
-      <c r="H886" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20260715</t>
-        </is>
-      </c>
-      <c r="I886" t="inlineStr">
-        <is>
-          <t xml:space="preserve">전남광주통합특별시　광산구　무진대로　２６１　（우산동）　５층　　　　　　　　　　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="J886" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       </t>
-        </is>
-      </c>
-    </row>
-    <row r="887">
-      <c r="A887" t="inlineStr">
-        <is>
-          <t xml:space="preserve">변경    </t>
-        </is>
-      </c>
-      <c r="B887" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0102209</t>
-        </is>
-      </c>
-      <c r="C887" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ＮＨ농협은행　　　　</t>
-        </is>
-      </c>
-      <c r="D887" t="inlineStr">
-        <is>
-          <t xml:space="preserve">송도금융센터　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="E887" t="inlineStr">
-        <is>
-          <t xml:space="preserve">032  858  0021 </t>
-        </is>
-      </c>
-      <c r="F887" t="inlineStr">
-        <is>
-          <t xml:space="preserve">032  858  0023 </t>
-        </is>
-      </c>
-      <c r="G887" t="inlineStr">
-        <is>
-          <t xml:space="preserve">22013 </t>
-        </is>
-      </c>
-      <c r="H887" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20260715</t>
-        </is>
-      </c>
-      <c r="I887" t="inlineStr">
-        <is>
-          <t xml:space="preserve">인천광역시　연수구　하모니로１７７번길　４９　（송도동）　　　　　　　　　　　　　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="J887" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       </t>
-        </is>
-      </c>
-    </row>
-    <row r="888">
-      <c r="A888" t="inlineStr">
-        <is>
-          <t xml:space="preserve">변경    </t>
-        </is>
-      </c>
-      <c r="B888" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0466194</t>
-        </is>
-      </c>
-      <c r="C888" t="inlineStr">
-        <is>
-          <t xml:space="preserve">새마을금고　　　　　</t>
-        </is>
-      </c>
-      <c r="D888" t="inlineStr">
-        <is>
-          <t xml:space="preserve">김천대신　　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="E888" t="inlineStr">
-        <is>
-          <t xml:space="preserve">054  433  5462 </t>
-        </is>
-      </c>
-      <c r="F888" t="inlineStr">
-        <is>
-          <t xml:space="preserve">054  437  5462 </t>
-        </is>
-      </c>
-      <c r="G888" t="inlineStr">
-        <is>
-          <t xml:space="preserve">39548 </t>
-        </is>
-      </c>
-      <c r="H888" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20260715</t>
-        </is>
-      </c>
-      <c r="I888" t="inlineStr">
-        <is>
-          <t xml:space="preserve">경북　김천시　부거리길　９　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="J888" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       </t>
-        </is>
-      </c>
-    </row>
-    <row r="889">
-      <c r="A889" t="inlineStr">
-        <is>
-          <t xml:space="preserve">변경    </t>
-        </is>
-      </c>
-      <c r="B889" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0490351</t>
-        </is>
-      </c>
-      <c r="C889" t="inlineStr">
-        <is>
-          <t xml:space="preserve">신협　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="D889" t="inlineStr">
-        <is>
-          <t xml:space="preserve">부산장우신협　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="E889" t="inlineStr">
-        <is>
-          <t xml:space="preserve">051  464  0019 </t>
-        </is>
-      </c>
-      <c r="F889" t="inlineStr">
-        <is>
-          <t xml:space="preserve">051  464  0266 </t>
-        </is>
-      </c>
-      <c r="G889" t="inlineStr">
-        <is>
-          <t xml:space="preserve">48814 </t>
-        </is>
-      </c>
-      <c r="H889" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20260715</t>
-        </is>
-      </c>
-      <c r="I889" t="inlineStr">
-        <is>
-          <t xml:space="preserve">부산광역시　동구　초량상로　９０－１　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="J889" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       </t>
-        </is>
-      </c>
-    </row>
-    <row r="890">
-      <c r="A890" t="inlineStr">
-        <is>
-          <t xml:space="preserve">변경    </t>
-        </is>
-      </c>
-      <c r="B890" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0877806</t>
-        </is>
-      </c>
-      <c r="C890" t="inlineStr">
-        <is>
-          <t xml:space="preserve">새마을금고　　　　　</t>
-        </is>
-      </c>
-      <c r="D890" t="inlineStr">
-        <is>
-          <t xml:space="preserve">김천대신금고　평화지점　　　　</t>
-        </is>
-      </c>
-      <c r="E890" t="inlineStr">
-        <is>
-          <t xml:space="preserve">054  434  1114 </t>
-        </is>
-      </c>
-      <c r="F890" t="inlineStr">
-        <is>
-          <t xml:space="preserve">054  435  5164 </t>
-        </is>
-      </c>
-      <c r="G890" t="inlineStr">
-        <is>
-          <t xml:space="preserve">39609 </t>
-        </is>
-      </c>
-      <c r="H890" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20260715</t>
-        </is>
-      </c>
-      <c r="I890" t="inlineStr">
-        <is>
-          <t xml:space="preserve">경상북도　김천시　김천로　１０６　（평화동）　　　　　　　　　　　　　　　　　　　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="J890" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       </t>
-        </is>
-      </c>
-    </row>
-    <row r="891">
-      <c r="A891" t="inlineStr">
-        <is>
-          <t xml:space="preserve">변경    </t>
-        </is>
-      </c>
-      <c r="B891" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0124708</t>
-        </is>
-      </c>
-      <c r="C891" t="inlineStr">
-        <is>
-          <t xml:space="preserve">농축협　　　　　　　</t>
-        </is>
-      </c>
-      <c r="D891" t="inlineStr">
-        <is>
-          <t xml:space="preserve">보성농협　　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="E891" t="inlineStr">
-        <is>
-          <t xml:space="preserve">061  850  7800 </t>
-        </is>
-      </c>
-      <c r="F891" t="inlineStr">
-        <is>
-          <t xml:space="preserve">061  853  6665 </t>
-        </is>
-      </c>
-      <c r="G891" t="inlineStr">
-        <is>
-          <t xml:space="preserve">59458 </t>
-        </is>
-      </c>
-      <c r="H891" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20260714</t>
-        </is>
-      </c>
-      <c r="I891" t="inlineStr">
-        <is>
-          <t xml:space="preserve">전남광주통합특별시　보성군　보성읍　현충로　９２－２０　　　　　　　　　　　　　　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="J891" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       </t>
-        </is>
-      </c>
-    </row>
-    <row r="892">
-      <c r="A892" t="inlineStr">
-        <is>
-          <t xml:space="preserve">변경    </t>
-        </is>
-      </c>
-      <c r="B892" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0129871</t>
-        </is>
-      </c>
-      <c r="C892" t="inlineStr">
-        <is>
-          <t xml:space="preserve">농축협　　　　　　　</t>
-        </is>
-      </c>
-      <c r="D892" t="inlineStr">
-        <is>
-          <t xml:space="preserve">중구농협　　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="E892" t="inlineStr">
-        <is>
-          <t xml:space="preserve">032  746  0989 </t>
-        </is>
-      </c>
-      <c r="F892" t="inlineStr">
-        <is>
-          <t xml:space="preserve">032  746  5078 </t>
-        </is>
-      </c>
-      <c r="G892" t="inlineStr">
-        <is>
-          <t xml:space="preserve">23249 </t>
-        </is>
-      </c>
-      <c r="H892" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20260714</t>
-        </is>
-      </c>
-      <c r="I892" t="inlineStr">
-        <is>
-          <t xml:space="preserve">인천광역시　영종구　운남로　１６６　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="J892" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       </t>
-        </is>
-      </c>
-    </row>
-    <row r="893">
-      <c r="A893" t="inlineStr">
-        <is>
-          <t xml:space="preserve">변경    </t>
-        </is>
-      </c>
-      <c r="B893" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0134468</t>
-        </is>
-      </c>
-      <c r="C893" t="inlineStr">
-        <is>
-          <t xml:space="preserve">농축협　　　　　　　</t>
-        </is>
-      </c>
-      <c r="D893" t="inlineStr">
-        <is>
-          <t xml:space="preserve">서광주　화정　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="E893" t="inlineStr">
-        <is>
-          <t xml:space="preserve">062  372  0421 </t>
-        </is>
-      </c>
-      <c r="F893" t="inlineStr">
-        <is>
-          <t xml:space="preserve">062  373  0408 </t>
-        </is>
-      </c>
-      <c r="G893" t="inlineStr">
-        <is>
-          <t xml:space="preserve">62026 </t>
-        </is>
-      </c>
-      <c r="H893" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20260714</t>
-        </is>
-      </c>
-      <c r="I893" t="inlineStr">
-        <is>
-          <t xml:space="preserve">전남광주통합특별시　서구　염화로　８１　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="J893" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       </t>
-        </is>
-      </c>
-    </row>
-    <row r="894">
-      <c r="A894" t="inlineStr">
-        <is>
-          <t xml:space="preserve">변경    </t>
-        </is>
-      </c>
-      <c r="B894" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0141794</t>
-        </is>
-      </c>
-      <c r="C894" t="inlineStr">
-        <is>
-          <t xml:space="preserve">농축협　　　　　　　</t>
-        </is>
-      </c>
-      <c r="D894" t="inlineStr">
-        <is>
-          <t xml:space="preserve">중구　용유　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="E894" t="inlineStr">
-        <is>
-          <t xml:space="preserve">032  746  3008 </t>
-        </is>
-      </c>
-      <c r="F894" t="inlineStr">
-        <is>
-          <t xml:space="preserve">032  746  9894 </t>
-        </is>
-      </c>
-      <c r="G894" t="inlineStr">
-        <is>
-          <t xml:space="preserve">23360 </t>
-        </is>
-      </c>
-      <c r="H894" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20260714</t>
-        </is>
-      </c>
-      <c r="I894" t="inlineStr">
-        <is>
-          <t xml:space="preserve">인천광역시　영종구　마시란로　３１４－１６　　　　　　　　　　　　　　　　　　　　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="J894" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       </t>
-        </is>
-      </c>
-    </row>
-    <row r="895">
-      <c r="A895" t="inlineStr">
-        <is>
-          <t xml:space="preserve">변경    </t>
-        </is>
-      </c>
-      <c r="B895" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0151153</t>
-        </is>
-      </c>
-      <c r="C895" t="inlineStr">
-        <is>
-          <t xml:space="preserve">농축협　　　　　　　</t>
-        </is>
-      </c>
-      <c r="D895" t="inlineStr">
-        <is>
-          <t xml:space="preserve">중구　하인천　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="E895" t="inlineStr">
-        <is>
-          <t xml:space="preserve">032  763  4602 </t>
-        </is>
-      </c>
-      <c r="F895" t="inlineStr">
-        <is>
-          <t xml:space="preserve">032  772  7353 </t>
-        </is>
-      </c>
-      <c r="G895" t="inlineStr">
-        <is>
-          <t xml:space="preserve">22312 </t>
-        </is>
-      </c>
-      <c r="H895" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20260714</t>
-        </is>
-      </c>
-      <c r="I895" t="inlineStr">
-        <is>
-          <t xml:space="preserve">인천광역시　제물포구　차이나타운로４４번길　３１－１３　　　　　　　　　　　　　　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="J895" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       </t>
-        </is>
-      </c>
-    </row>
-    <row r="896">
-      <c r="A896" t="inlineStr">
-        <is>
-          <t xml:space="preserve">변경    </t>
-        </is>
-      </c>
-      <c r="B896" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0156323</t>
-        </is>
-      </c>
-      <c r="C896" t="inlineStr">
-        <is>
-          <t xml:space="preserve">농축협　　　　　　　</t>
-        </is>
-      </c>
-      <c r="D896" t="inlineStr">
-        <is>
-          <t xml:space="preserve">순천원예농협　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="E896" t="inlineStr">
-        <is>
-          <t xml:space="preserve">061  746  7500 </t>
-        </is>
-      </c>
-      <c r="F896" t="inlineStr">
-        <is>
-          <t xml:space="preserve">061  746  9530 </t>
-        </is>
-      </c>
-      <c r="G896" t="inlineStr">
-        <is>
-          <t xml:space="preserve">57996 </t>
-        </is>
-      </c>
-      <c r="H896" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20260714</t>
-        </is>
-      </c>
-      <c r="I896" t="inlineStr">
-        <is>
-          <t xml:space="preserve">전남광주통합특별시　순천시　남산로　４６　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="J896" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       </t>
-        </is>
-      </c>
-    </row>
-    <row r="897">
-      <c r="A897" t="inlineStr">
-        <is>
-          <t xml:space="preserve">변경    </t>
-        </is>
-      </c>
-      <c r="B897" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0159278</t>
-        </is>
-      </c>
-      <c r="C897" t="inlineStr">
-        <is>
-          <t xml:space="preserve">농축협　　　　　　　</t>
-        </is>
-      </c>
-      <c r="D897" t="inlineStr">
-        <is>
-          <t xml:space="preserve">중구　공항신도시　　　　　　　</t>
-        </is>
-      </c>
-      <c r="E897" t="inlineStr">
-        <is>
-          <t xml:space="preserve">032  752  1414 </t>
-        </is>
-      </c>
-      <c r="F897" t="inlineStr">
-        <is>
-          <t xml:space="preserve">032  752  1420 </t>
-        </is>
-      </c>
-      <c r="G897" t="inlineStr">
-        <is>
-          <t xml:space="preserve">23211 </t>
-        </is>
-      </c>
-      <c r="H897" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20260714</t>
-        </is>
-      </c>
-      <c r="I897" t="inlineStr">
-        <is>
-          <t xml:space="preserve">인천광역시　영종구　신도시남로１４２번길　６　（운서동）　　　　　　　　　　　　　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="J897" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       </t>
-        </is>
-      </c>
-    </row>
-    <row r="898">
-      <c r="A898" t="inlineStr">
-        <is>
-          <t xml:space="preserve">변경    </t>
-        </is>
-      </c>
-      <c r="B898" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0180328</t>
-        </is>
-      </c>
-      <c r="C898" t="inlineStr">
-        <is>
-          <t xml:space="preserve">농축협　　　　　　　</t>
-        </is>
-      </c>
-      <c r="D898" t="inlineStr">
-        <is>
-          <t xml:space="preserve">중구　하늘도시　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="E898" t="inlineStr">
-        <is>
-          <t xml:space="preserve">032  746  1441 </t>
-        </is>
-      </c>
-      <c r="F898" t="inlineStr">
-        <is>
-          <t xml:space="preserve">032  746  1551 </t>
-        </is>
-      </c>
-      <c r="G898" t="inlineStr">
-        <is>
-          <t xml:space="preserve">23303 </t>
-        </is>
-      </c>
-      <c r="H898" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20260714</t>
-        </is>
-      </c>
-      <c r="I898" t="inlineStr">
-        <is>
-          <t xml:space="preserve">인천광역시　영종구　하늘중앙로１９５번길　１４　　　　　　　　　　　　　　　　　　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="J898" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       </t>
-        </is>
-      </c>
-    </row>
-    <row r="899">
-      <c r="A899" t="inlineStr">
-        <is>
-          <t xml:space="preserve">신규    </t>
-        </is>
-      </c>
-      <c r="B899" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0508670</t>
-        </is>
-      </c>
-      <c r="C899" t="inlineStr">
-        <is>
-          <t xml:space="preserve">저축은행　　　　　　</t>
-        </is>
-      </c>
-      <c r="D899" t="inlineStr">
-        <is>
-          <t xml:space="preserve">참　　　　　경영관리팀　　　　</t>
-        </is>
-      </c>
-      <c r="E899" t="inlineStr">
-        <is>
-          <t xml:space="preserve">053  720  7300 </t>
-        </is>
-      </c>
-      <c r="F899" t="inlineStr">
-        <is>
-          <t xml:space="preserve">053  720  7407 </t>
-        </is>
-      </c>
-      <c r="G899" t="inlineStr">
-        <is>
-          <t xml:space="preserve">42028 </t>
-        </is>
-      </c>
-      <c r="H899" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20260714</t>
-        </is>
-      </c>
-      <c r="I899" t="inlineStr">
-        <is>
-          <t xml:space="preserve">대구광역시　수성구　달구벌대로　２４２１　（범어동）　２층　　　　　　　　　　　　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="J899" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       </t>
-        </is>
-      </c>
-    </row>
-    <row r="900">
-      <c r="A900" t="inlineStr">
-        <is>
-          <t xml:space="preserve">신규    </t>
-        </is>
-      </c>
-      <c r="B900" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0508683</t>
-        </is>
-      </c>
-      <c r="C900" t="inlineStr">
-        <is>
-          <t xml:space="preserve">저축은행　　　　　　</t>
-        </is>
-      </c>
-      <c r="D900" t="inlineStr">
-        <is>
-          <t xml:space="preserve">참　　　　　경영전략팀　　　　</t>
-        </is>
-      </c>
-      <c r="E900" t="inlineStr">
-        <is>
-          <t xml:space="preserve">053  720  7300 </t>
-        </is>
-      </c>
-      <c r="F900" t="inlineStr">
-        <is>
-          <t xml:space="preserve">053  720  7400 </t>
-        </is>
-      </c>
-      <c r="G900" t="inlineStr">
-        <is>
-          <t xml:space="preserve">42028 </t>
-        </is>
-      </c>
-      <c r="H900" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20260714</t>
-        </is>
-      </c>
-      <c r="I900" t="inlineStr">
-        <is>
-          <t xml:space="preserve">대구광역시　수성구　달구벌대로　２４２１　（범어동）　２층　　　　　　　　　　　　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="J900" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       </t>
-        </is>
-      </c>
-    </row>
-    <row r="901">
-      <c r="A901" t="inlineStr">
-        <is>
-          <t xml:space="preserve">신규    </t>
-        </is>
-      </c>
-      <c r="B901" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0508696</t>
-        </is>
-      </c>
-      <c r="C901" t="inlineStr">
-        <is>
-          <t xml:space="preserve">저축은행　　　　　　</t>
-        </is>
-      </c>
-      <c r="D901" t="inlineStr">
-        <is>
-          <t xml:space="preserve">참　　　　　수신영업팀　　　　</t>
-        </is>
-      </c>
-      <c r="E901" t="inlineStr">
-        <is>
-          <t xml:space="preserve">053  720  7300 </t>
-        </is>
-      </c>
-      <c r="F901" t="inlineStr">
-        <is>
-          <t xml:space="preserve">053  720  7405 </t>
-        </is>
-      </c>
-      <c r="G901" t="inlineStr">
-        <is>
-          <t xml:space="preserve">42028 </t>
-        </is>
-      </c>
-      <c r="H901" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20260714</t>
-        </is>
-      </c>
-      <c r="I901" t="inlineStr">
-        <is>
-          <t xml:space="preserve">대구광역시　수성구　달구벌대로　２４２１　（범어동）　２층　　　　　　　　　　　　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="J901" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       </t>
-        </is>
-      </c>
-    </row>
-    <row r="902">
-      <c r="A902" t="inlineStr">
-        <is>
-          <t xml:space="preserve">신규    </t>
-        </is>
-      </c>
-      <c r="B902" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0508706</t>
-        </is>
-      </c>
-      <c r="C902" t="inlineStr">
-        <is>
-          <t xml:space="preserve">저축은행　　　　　　</t>
-        </is>
-      </c>
-      <c r="D902" t="inlineStr">
-        <is>
-          <t xml:space="preserve">참　　　　　기업금융１팀　　　</t>
-        </is>
-      </c>
-      <c r="E902" t="inlineStr">
-        <is>
-          <t xml:space="preserve">053  720  7300 </t>
-        </is>
-      </c>
-      <c r="F902" t="inlineStr">
-        <is>
-          <t xml:space="preserve">053  720  7402 </t>
-        </is>
-      </c>
-      <c r="G902" t="inlineStr">
-        <is>
-          <t xml:space="preserve">42028 </t>
-        </is>
-      </c>
-      <c r="H902" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20260714</t>
-        </is>
-      </c>
-      <c r="I902" t="inlineStr">
-        <is>
-          <t xml:space="preserve">대구광역시　수성구　달구벌대로　２４２１　（범어동）　２층　　　　　　　　　　　　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="J902" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       </t>
-        </is>
-      </c>
-    </row>
-    <row r="903">
-      <c r="A903" t="inlineStr">
-        <is>
-          <t xml:space="preserve">신규    </t>
-        </is>
-      </c>
-      <c r="B903" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0508719</t>
-        </is>
-      </c>
-      <c r="C903" t="inlineStr">
-        <is>
-          <t xml:space="preserve">저축은행　　　　　　</t>
-        </is>
-      </c>
-      <c r="D903" t="inlineStr">
-        <is>
-          <t xml:space="preserve">참　　　　　기업금융２팀　　　</t>
-        </is>
-      </c>
-      <c r="E903" t="inlineStr">
-        <is>
-          <t xml:space="preserve">053  720  7300 </t>
-        </is>
-      </c>
-      <c r="F903" t="inlineStr">
-        <is>
-          <t xml:space="preserve">053  720  7404 </t>
-        </is>
-      </c>
-      <c r="G903" t="inlineStr">
-        <is>
-          <t xml:space="preserve">42028 </t>
-        </is>
-      </c>
-      <c r="H903" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20260714</t>
-        </is>
-      </c>
-      <c r="I903" t="inlineStr">
-        <is>
-          <t xml:space="preserve">대구광역시　수성구　달구벌대로　２４２１　（범어동）　２층　　　　　　　　　　　　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="J903" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       </t>
-        </is>
-      </c>
-    </row>
-    <row r="904">
-      <c r="A904" t="inlineStr">
-        <is>
-          <t xml:space="preserve">신규    </t>
-        </is>
-      </c>
-      <c r="B904" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0508722</t>
-        </is>
-      </c>
-      <c r="C904" t="inlineStr">
-        <is>
-          <t xml:space="preserve">저축은행　　　　　　</t>
-        </is>
-      </c>
-      <c r="D904" t="inlineStr">
-        <is>
-          <t xml:space="preserve">참　　　　　여신관리팀　　　　</t>
-        </is>
-      </c>
-      <c r="E904" t="inlineStr">
-        <is>
-          <t xml:space="preserve">053  720  7300 </t>
-        </is>
-      </c>
-      <c r="F904" t="inlineStr">
-        <is>
-          <t xml:space="preserve">053  720  7402 </t>
-        </is>
-      </c>
-      <c r="G904" t="inlineStr">
-        <is>
-          <t xml:space="preserve">42028 </t>
-        </is>
-      </c>
-      <c r="H904" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20260714</t>
-        </is>
-      </c>
-      <c r="I904" t="inlineStr">
-        <is>
-          <t xml:space="preserve">대구광역시　수성구　달구벌대로　２４２１　（범어동）　２층　　　　　　　　　　　　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="J904" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       </t>
-        </is>
-      </c>
-    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>